<commit_message>
feat(F-NAR-019): polish TREE-DIF-024 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-024.xlsx
+++ b/stories/arbres/TREE-DIF-024.xlsx
@@ -17545,7 +17545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17651,6 +17651,13 @@
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>